<commit_message>
refactor: inclusão de melhorias e atualização do horário
</commit_message>
<xml_diff>
--- a/scripts/input/Ocupacao.xlsx
+++ b/scripts/input/Ocupacao.xlsx
@@ -1,45 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carol\Documents\salas-cefet\scripts\input\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D36CBF-7C18-4AEA-9B59-F5F4E29FBEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="10500" xr2:uid="{C3C8C009-1FF4-4949-AB30-D4C8428C6CB3}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet state="visible" name="Planilha1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="IvEvuksAwlF6a9zvjY8QmKabH1fIG2S4DjwBxkmDlwk="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="29">
   <si>
     <t>sala</t>
   </si>
@@ -131,22 +108,33 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <fonts count="5">
     <font>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -154,59 +142,56 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="lightGray"/>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="5">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Sheets">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
@@ -230,113 +215,19 @@
         <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="467886"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Sheets">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Aptos Narrow"/>
+        <a:ea typeface="Aptos Narrow"/>
+        <a:cs typeface="Aptos Narrow"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Aptos Narrow"/>
+        <a:ea typeface="Aptos Narrow"/>
+        <a:cs typeface="Aptos Narrow"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -398,6 +289,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -406,13 +304,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -477,45 +368,21 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EE9623-4962-4105-AFCB-86FDFF7C4F1F}">
-  <dimension ref="A1:T196"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <pageSetUpPr/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="40.33203125" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="40.38"/>
+    <col customWidth="1" min="2" max="26" width="8.63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -577,9 +444,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2">
-        <v>7</v>
+        <v>7.0</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>20</v>
@@ -609,21 +476,31 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
+      <c r="N2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2">
-        <v>7</v>
+        <v>7.0</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>20</v>
@@ -650,14 +527,24 @@
         <v>22</v>
       </c>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
+      <c r="K3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q3" s="2" t="s">
         <v>22</v>
       </c>
@@ -671,9 +558,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2">
-        <v>7</v>
+        <v>7.0</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>20</v>
@@ -703,11 +590,13 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="N4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="2"/>
       <c r="Q4" s="2" t="s">
         <v>22</v>
       </c>
@@ -721,9 +610,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2">
-        <v>7</v>
+        <v>7.0</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>20</v>
@@ -763,9 +652,7 @@
         <v>22</v>
       </c>
       <c r="O5" s="2"/>
-      <c r="P5" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P5" s="2"/>
       <c r="Q5" s="2" t="s">
         <v>22</v>
       </c>
@@ -779,9 +666,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2">
-        <v>7</v>
+        <v>7.0</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>20</v>
@@ -820,16 +707,12 @@
       <c r="R6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+    </row>
+    <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2">
-        <v>7</v>
+        <v>7.0</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>20</v>
@@ -859,9 +742,9 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2">
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>20</v>
@@ -881,8 +764,12 @@
       <c r="G8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="H8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
         <v>22</v>
@@ -897,7 +784,9 @@
         <v>22</v>
       </c>
       <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
+      <c r="P8" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q8" s="2" t="s">
         <v>22</v>
       </c>
@@ -911,9 +800,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2">
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>20</v>
@@ -951,9 +840,7 @@
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P9" s="2"/>
       <c r="Q9" s="2" t="s">
         <v>22</v>
       </c>
@@ -967,9 +854,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2">
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>20</v>
@@ -1001,9 +888,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P10" s="2"/>
       <c r="Q10" s="2" t="s">
         <v>22</v>
       </c>
@@ -1017,9 +902,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2">
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>20</v>
@@ -1067,9 +952,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2">
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>20</v>
@@ -1108,16 +993,12 @@
       <c r="R12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+    </row>
+    <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2">
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>20</v>
@@ -1143,9 +1024,9 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2">
-        <v>16</v>
+        <v>16.0</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>20</v>
@@ -1153,8 +1034,12 @@
       <c r="C14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="D14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="F14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1166,24 +1051,32 @@
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
       <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
+      <c r="N14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="T14" s="2"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2">
-        <v>16</v>
+        <v>16.0</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>20</v>
@@ -1237,9 +1130,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2">
-        <v>16</v>
+        <v>16.0</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>20</v>
@@ -1269,10 +1162,16 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2" t="s">
+      <c r="N16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="R16" s="2" t="s">
@@ -1285,9 +1184,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2">
-        <v>16</v>
+        <v>16.0</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>20</v>
@@ -1329,9 +1228,9 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2">
-        <v>16</v>
+        <v>16.0</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>20</v>
@@ -1354,7 +1253,7 @@
       <c r="H18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="3" t="s">
         <v>22</v>
       </c>
       <c r="J18" s="2"/>
@@ -1363,15 +1262,25 @@
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2">
-        <v>16</v>
+        <v>16.0</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>20</v>
@@ -1397,9 +1306,9 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2">
-        <v>17</v>
+        <v>17.0</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>20</v>
@@ -1423,21 +1332,11 @@
         <v>22</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
       <c r="Q20" s="2" t="s">
@@ -1446,12 +1345,16 @@
       <c r="R20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2"/>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T20" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="2">
-        <v>17</v>
+        <v>17.0</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>20</v>
@@ -1477,9 +1380,7 @@
       <c r="I21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="J21" s="2"/>
       <c r="K21" s="2" t="s">
         <v>22</v>
       </c>
@@ -1509,9 +1410,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="2">
-        <v>17</v>
+        <v>17.0</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>20</v>
@@ -1539,10 +1440,18 @@
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+      <c r="L22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O22" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="P22" s="2" t="s">
         <v>22</v>
       </c>
@@ -1559,9 +1468,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="2">
-        <v>17</v>
+        <v>17.0</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>20</v>
@@ -1587,9 +1496,7 @@
       <c r="I23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="J23" s="2"/>
       <c r="K23" s="2" t="s">
         <v>22</v>
       </c>
@@ -1603,19 +1510,17 @@
         <v>22</v>
       </c>
       <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
+      <c r="P23" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
-      <c r="S23" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T23" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
+    </row>
+    <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="2">
-        <v>17</v>
+        <v>17.0</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>20</v>
@@ -1661,9 +1566,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="2">
-        <v>17</v>
+        <v>17.0</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>20</v>
@@ -1693,9 +1598,9 @@
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="2">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>20</v>
@@ -1703,7 +1608,7 @@
       <c r="C26" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E26" s="2" t="s">
@@ -1735,9 +1640,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="2">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>20</v>
@@ -1751,8 +1656,12 @@
       <c r="E27" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="F27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="H27" s="2" t="s">
         <v>22</v>
       </c>
@@ -1761,14 +1670,14 @@
       </c>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="L27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N27" s="2"/>
+      <c r="O27" s="2"/>
       <c r="P27" s="2"/>
       <c r="Q27" s="2" t="s">
         <v>22</v>
@@ -1783,9 +1692,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="2">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>20</v>
@@ -1815,12 +1724,8 @@
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
-      <c r="N28" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
       <c r="P28" s="2" t="s">
         <v>22</v>
       </c>
@@ -1830,12 +1735,16 @@
       <c r="R28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2"/>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25" customHeight="1">
       <c r="A29" s="2">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>20</v>
@@ -1875,9 +1784,7 @@
         <v>22</v>
       </c>
       <c r="O29" s="2"/>
-      <c r="P29" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P29" s="2"/>
       <c r="Q29" s="2" t="s">
         <v>22</v>
       </c>
@@ -1891,9 +1798,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="2">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>20</v>
@@ -1926,18 +1833,18 @@
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
-      <c r="Q30" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R30" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="2">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>20</v>
@@ -1963,9 +1870,9 @@
       <c r="S31" s="2"/>
       <c r="T31" s="2"/>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" ht="14.25" customHeight="1">
       <c r="A32" s="2">
-        <v>31</v>
+        <v>31.0</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>20</v>
@@ -2003,17 +1910,15 @@
       <c r="Q32" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R32" s="2"/>
-      <c r="S32" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T32" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R32" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S32" s="2"/>
+      <c r="T32" s="2"/>
+    </row>
+    <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="2">
-        <v>31</v>
+        <v>31.0</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>20</v>
@@ -2051,19 +1956,25 @@
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
+      <c r="P33" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q33" s="2" t="s">
         <v>22</v>
       </c>
       <c r="R33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S33" s="2"/>
-      <c r="T33" s="2"/>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S33" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T33" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="2">
-        <v>31</v>
+        <v>31.0</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>20</v>
@@ -2097,9 +2008,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="2">
-        <v>31</v>
+        <v>31.0</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>20</v>
@@ -2135,7 +2046,9 @@
         <v>22</v>
       </c>
       <c r="O35" s="2"/>
-      <c r="P35" s="2"/>
+      <c r="P35" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q35" s="2" t="s">
         <v>22</v>
       </c>
@@ -2149,9 +2062,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="2">
-        <v>31</v>
+        <v>31.0</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>20</v>
@@ -2184,14 +2097,18 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-      <c r="R36" s="2"/>
+      <c r="Q36" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="2">
-        <v>31</v>
+        <v>31.0</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>20</v>
@@ -2217,9 +2134,9 @@
       <c r="S37" s="2"/>
       <c r="T37" s="2"/>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" ht="14.25" customHeight="1">
       <c r="A38" s="2">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>20</v>
@@ -2251,15 +2168,21 @@
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
-      <c r="P38" s="2"/>
-      <c r="Q38" s="2"/>
-      <c r="R38" s="2"/>
+      <c r="P38" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S38" s="2"/>
       <c r="T38" s="2"/>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="2">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>20</v>
@@ -2297,15 +2220,21 @@
         <v>22</v>
       </c>
       <c r="O39" s="2"/>
-      <c r="P39" s="2"/>
-      <c r="Q39" s="2"/>
-      <c r="R39" s="2"/>
+      <c r="P39" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q39" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R39" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S39" s="2"/>
       <c r="T39" s="2"/>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="2">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>20</v>
@@ -2337,21 +2266,15 @@
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
-      <c r="P40" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q40" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R40" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P40" s="2"/>
+      <c r="Q40" s="2"/>
+      <c r="R40" s="2"/>
       <c r="S40" s="2"/>
       <c r="T40" s="2"/>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" ht="14.25" customHeight="1">
       <c r="A41" s="2">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>20</v>
@@ -2384,18 +2307,14 @@
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
-      <c r="Q41" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="Q41" s="2"/>
+      <c r="R41" s="2"/>
       <c r="S41" s="2"/>
       <c r="T41" s="2"/>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="2">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>20</v>
@@ -2433,9 +2352,9 @@
       <c r="S42" s="2"/>
       <c r="T42" s="2"/>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="2">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>20</v>
@@ -2461,9 +2380,9 @@
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" ht="14.25" customHeight="1">
       <c r="A44" s="2">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>20</v>
@@ -2471,20 +2390,20 @@
       <c r="C44" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
       <c r="F44" s="2" t="s">
         <v>22</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
+      <c r="H44" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J44" s="2"/>
       <c r="K44" s="2" t="s">
         <v>22</v>
@@ -2493,11 +2412,13 @@
         <v>22</v>
       </c>
       <c r="M44" s="2"/>
-      <c r="N44" s="2"/>
-      <c r="O44" s="2"/>
-      <c r="P44" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="N44" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P44" s="2"/>
       <c r="Q44" s="2" t="s">
         <v>22</v>
       </c>
@@ -2507,9 +2428,9 @@
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="2">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>20</v>
@@ -2519,12 +2440,8 @@
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
-      <c r="F45" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
       <c r="H45" s="2" t="s">
         <v>22</v>
       </c>
@@ -2537,15 +2454,23 @@
       <c r="K45" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
+      <c r="L45" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O45" s="2"/>
-      <c r="P45" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
+      <c r="P45" s="2"/>
+      <c r="Q45" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R45" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S45" s="2" t="s">
         <v>22</v>
       </c>
@@ -2553,9 +2478,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="2">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>20</v>
@@ -2575,25 +2500,21 @@
       <c r="G46" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
+      <c r="H46" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
-      <c r="N46" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O46" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
       <c r="P46" s="2"/>
-      <c r="Q46" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R46" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" s="2"/>
       <c r="S46" s="2" t="s">
         <v>22</v>
       </c>
@@ -2601,9 +2522,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" ht="14.25" customHeight="1">
       <c r="A47" s="2">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>20</v>
@@ -2625,25 +2546,37 @@
       <c r="I47" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
-      <c r="N47" s="2"/>
+      <c r="J47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N47" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O47" s="2"/>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="R47" s="2"/>
-      <c r="S47" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T47" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S47" s="2"/>
+      <c r="T47" s="2"/>
+    </row>
+    <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="2">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>20</v>
@@ -2663,12 +2596,8 @@
       <c r="G48" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
@@ -2678,22 +2607,14 @@
       <c r="P48" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Q48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T48" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q48" s="2"/>
+      <c r="R48" s="2"/>
+      <c r="S48" s="2"/>
+      <c r="T48" s="2"/>
+    </row>
+    <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="2">
-        <v>34</v>
+        <v>34.0</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>20</v>
@@ -2719,9 +2640,9 @@
       <c r="S49" s="2"/>
       <c r="T49" s="2"/>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="50" ht="14.25" customHeight="1">
       <c r="A50" s="2">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>20</v>
@@ -2739,21 +2660,35 @@
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
-      <c r="N50" s="2"/>
+      <c r="J50" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L50" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M50" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N50" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
-      <c r="Q50" s="2"/>
-      <c r="R50" s="2"/>
+      <c r="Q50" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R50" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S50" s="2"/>
       <c r="T50" s="2"/>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="2">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>20</v>
@@ -2801,9 +2736,9 @@
       <c r="S51" s="2"/>
       <c r="T51" s="2"/>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="2">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>20</v>
@@ -2823,7 +2758,9 @@
       <c r="M52" s="2"/>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
-      <c r="P52" s="2"/>
+      <c r="P52" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q52" s="2" t="s">
         <v>22</v>
       </c>
@@ -2833,9 +2770,9 @@
       <c r="S52" s="2"/>
       <c r="T52" s="2"/>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="53" ht="14.25" customHeight="1">
       <c r="A53" s="2">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>20</v>
@@ -2875,7 +2812,9 @@
         <v>22</v>
       </c>
       <c r="O53" s="2"/>
-      <c r="P53" s="2"/>
+      <c r="P53" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q53" s="2" t="s">
         <v>22</v>
       </c>
@@ -2889,9 +2828,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="2">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>20</v>
@@ -2923,23 +2862,17 @@
       <c r="M54" s="2"/>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
-      <c r="P54" s="2"/>
-      <c r="Q54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T54" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P54" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q54" s="2"/>
+      <c r="R54" s="2"/>
+      <c r="S54" s="2"/>
+      <c r="T54" s="2"/>
+    </row>
+    <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="2">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>20</v>
@@ -2965,9 +2898,9 @@
       <c r="S55" s="2"/>
       <c r="T55" s="2"/>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="56" ht="14.25" customHeight="1">
       <c r="A56" s="2">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>20</v>
@@ -2975,51 +2908,45 @@
       <c r="C56" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
       <c r="J56" s="2" t="s">
         <v>22</v>
       </c>
       <c r="K56" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L56" s="2"/>
-      <c r="M56" s="2"/>
+      <c r="L56" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M56" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="N56" s="2" t="s">
         <v>22</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="P56" s="2"/>
-      <c r="Q56" s="2"/>
-      <c r="R56" s="2"/>
-      <c r="S56" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T56" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P56" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q56" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R56" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S56" s="2"/>
+      <c r="T56" s="2"/>
+    </row>
+    <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="2">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>20</v>
@@ -3027,18 +2954,10 @@
       <c r="C57" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
       <c r="H57" s="2" t="s">
         <v>22</v>
       </c>
@@ -3056,12 +2975,16 @@
       <c r="N57" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="O57" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="P57" s="2"/>
-      <c r="Q57" s="2"/>
-      <c r="R57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q57" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R57" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S57" s="2" t="s">
         <v>22</v>
       </c>
@@ -3069,9 +2992,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="2">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>20</v>
@@ -3079,8 +3002,12 @@
       <c r="C58" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
+      <c r="D58" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="F58" s="2" t="s">
         <v>22</v>
       </c>
@@ -3095,23 +3022,21 @@
       </c>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
-      <c r="L58" s="2"/>
-      <c r="M58" s="2"/>
-      <c r="N58" s="2" t="s">
+      <c r="L58" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M58" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N58" s="3" t="s">
         <v>22</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="P58" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q58" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R58" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P58" s="2"/>
+      <c r="Q58" s="2"/>
+      <c r="R58" s="2"/>
       <c r="S58" s="2" t="s">
         <v>22</v>
       </c>
@@ -3119,9 +3044,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="59" ht="14.25" customHeight="1">
       <c r="A59" s="2">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>20</v>
@@ -3135,20 +3060,12 @@
       <c r="E59" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F59" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
-      <c r="J59" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K59" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
       <c r="L59" s="2" t="s">
         <v>22</v>
       </c>
@@ -3158,9 +3075,7 @@
       <c r="N59" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="O59" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="O59" s="2"/>
       <c r="P59" s="2" t="s">
         <v>22</v>
       </c>
@@ -3170,16 +3085,12 @@
       <c r="R59" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S59" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T59" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S59" s="2"/>
+      <c r="T59" s="2"/>
+    </row>
+    <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="2">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>20</v>
@@ -3187,22 +3098,14 @@
       <c r="C60" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H60" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q60" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R60" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="H60" s="2"/>
+      <c r="I60" s="2"/>
+      <c r="Q60" s="2"/>
+      <c r="R60" s="2"/>
+    </row>
+    <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="2">
-        <v>37</v>
+        <v>37.0</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>20</v>
@@ -3215,9 +3118,9 @@
       <c r="Q61" s="2"/>
       <c r="R61" s="2"/>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="62" ht="14.25" customHeight="1">
       <c r="A62" s="2">
-        <v>39</v>
+        <v>39.0</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>20</v>
@@ -3243,16 +3146,33 @@
       <c r="I62" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S62" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T62" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="J62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="P62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="R62" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="S62" s="2"/>
+      <c r="T62" s="2"/>
+    </row>
+    <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="2">
-        <v>39</v>
+        <v>39.0</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>20</v>
@@ -3290,9 +3210,15 @@
       <c r="M63" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
-      <c r="P63" s="2"/>
+      <c r="N63" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O63" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P63" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="Q63" s="2" t="s">
         <v>22</v>
       </c>
@@ -3306,9 +3232,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="2">
-        <v>39</v>
+        <v>39.0</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>20</v>
@@ -3318,12 +3244,8 @@
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
-      <c r="F64" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G64" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="F64" s="2"/>
+      <c r="G64" s="2"/>
       <c r="H64" s="2" t="s">
         <v>22</v>
       </c>
@@ -3344,9 +3266,7 @@
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
-      <c r="P64" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P64" s="2"/>
       <c r="Q64" s="2" t="s">
         <v>22</v>
       </c>
@@ -3360,9 +3280,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" ht="14.25" customHeight="1">
       <c r="A65" s="2">
-        <v>39</v>
+        <v>39.0</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>20</v>
@@ -3390,23 +3310,21 @@
       <c r="K65" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L65" s="2"/>
-      <c r="M65" s="2"/>
+      <c r="L65" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M65" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="N65" s="2" t="s">
         <v>22</v>
       </c>
       <c r="O65" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="P65" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q65" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R65" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P65" s="2"/>
+      <c r="Q65" s="2"/>
+      <c r="R65" s="2"/>
       <c r="S65" s="2" t="s">
         <v>22</v>
       </c>
@@ -3414,9 +3332,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="2">
-        <v>39</v>
+        <v>39.0</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>20</v>
@@ -3424,41 +3342,25 @@
       <c r="C66" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I66" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+      <c r="G66" s="2"/>
+      <c r="H66" s="2"/>
+      <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
-      <c r="L66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N66" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O66" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="L66" s="2"/>
+      <c r="M66" s="2"/>
+      <c r="N66" s="2"/>
+      <c r="O66" s="2"/>
       <c r="P66" s="2"/>
-      <c r="Q66" s="2"/>
-      <c r="R66" s="2"/>
+      <c r="Q66" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R66" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="S66" s="2" t="s">
         <v>22</v>
       </c>
@@ -3466,9 +3368,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="2">
-        <v>39</v>
+        <v>39.0</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>20</v>
@@ -3494,9 +3396,9 @@
       <c r="S67" s="2"/>
       <c r="T67" s="2"/>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" ht="14.25" customHeight="1">
       <c r="A68" s="2">
-        <v>43</v>
+        <v>43.0</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>20</v>
@@ -3504,12 +3406,8 @@
       <c r="C68" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
       <c r="F68" s="2" t="s">
         <v>22</v>
       </c>
@@ -3532,25 +3430,19 @@
       <c r="M68" s="2"/>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
-      <c r="P68" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="P68" s="2"/>
       <c r="Q68" s="2" t="s">
         <v>22</v>
       </c>
       <c r="R68" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S68" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T68" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="S68" s="2"/>
+      <c r="T68" s="2"/>
+    </row>
+    <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="2">
-        <v>43</v>
+        <v>43.0</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>20</v>
@@ -3583,15 +3475,9 @@
       <c r="L69" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M69" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N69" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O69" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="M69" s="2"/>
+      <c r="N69" s="2"/>
+      <c r="O69" s="2"/>
       <c r="P69" s="2"/>
       <c r="Q69" s="2" t="s">
         <v>22</v>
@@ -3602,9 +3488,9 @@
       <c r="S69" s="2"/>
       <c r="T69" s="2"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="2">
-        <v>43</v>
+        <v>43.0</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>20</v>
@@ -3631,18 +3517,22 @@
         <v>22</v>
       </c>
       <c r="J70" s="2"/>
-      <c r="K70" s="2"/>
-      <c r="L70" s="2"/>
-      <c r="M70" s="2"/>
-      <c r="N70" s="2"/>
+      <c r="K70" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L70" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M70" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N70" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
-      <c r="Q70" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R70" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="Q70" s="2"/>
+      <c r="R70" s="2"/>
       <c r="S70" s="2" t="s">
         <v>22</v>
       </c>
@@ -3650,9 +3540,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" ht="14.25" customHeight="1">
       <c r="A71" s="2">
-        <v>43</v>
+        <v>43.0</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>20</v>
@@ -3660,8 +3550,12 @@
       <c r="C71" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
+      <c r="D71" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="F71" s="2" t="s">
         <v>22</v>
       </c>
@@ -3688,25 +3582,15 @@
         <v>22</v>
       </c>
       <c r="O71" s="2"/>
-      <c r="P71" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q71" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R71" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S71" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T71" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="P71" s="2"/>
+      <c r="Q71" s="2"/>
+      <c r="R71" s="2"/>
+      <c r="S71" s="2"/>
+      <c r="T71" s="2"/>
+    </row>
+    <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="2">
-        <v>43</v>
+        <v>43.0</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>20</v>
@@ -3726,31 +3610,35 @@
       <c r="G72" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H72" s="2"/>
-      <c r="I72" s="2"/>
+      <c r="H72" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J72" s="2"/>
-      <c r="K72" s="2"/>
-      <c r="L72" s="2"/>
-      <c r="M72" s="2"/>
-      <c r="N72" s="2"/>
+      <c r="K72" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L72" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M72" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N72" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
-      <c r="Q72" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R72" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S72" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T72" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q72" s="2"/>
+      <c r="R72" s="2"/>
+      <c r="S72" s="2"/>
+      <c r="T72" s="2"/>
+    </row>
+    <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="2">
-        <v>43</v>
+        <v>43.0</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>20</v>
@@ -3776,9 +3664,9 @@
       <c r="S73" s="2"/>
       <c r="T73" s="2"/>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" ht="14.25" customHeight="1">
       <c r="A74" s="2">
-        <v>46</v>
+        <v>46.0</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>20</v>
@@ -3798,17 +3686,17 @@
       <c r="G74" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
+      <c r="H74" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
       <c r="L74" s="2"/>
-      <c r="M74" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N74" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="M74" s="2"/>
+      <c r="N74" s="2"/>
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
       <c r="Q74" s="2"/>
@@ -3816,9 +3704,9 @@
       <c r="S74" s="2"/>
       <c r="T74" s="2"/>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="2">
-        <v>46</v>
+        <v>46.0</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>20</v>
@@ -3832,12 +3720,8 @@
       <c r="E75" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F75" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G75" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
       <c r="H75" s="2" t="s">
         <v>22</v>
       </c>
@@ -3851,8 +3735,12 @@
       <c r="L75" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M75" s="2"/>
-      <c r="N75" s="2"/>
+      <c r="M75" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N75" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
       <c r="Q75" s="2"/>
@@ -3860,9 +3748,9 @@
       <c r="S75" s="2"/>
       <c r="T75" s="2"/>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="2">
-        <v>46</v>
+        <v>46.0</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>20</v>
@@ -3889,24 +3777,28 @@
         <v>22</v>
       </c>
       <c r="J76" s="2"/>
-      <c r="K76" s="2"/>
-      <c r="L76" s="2"/>
-      <c r="M76" s="2"/>
-      <c r="N76" s="2"/>
+      <c r="K76" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L76" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M76" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N76" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
-      <c r="Q76" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R76" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="Q76" s="2"/>
+      <c r="R76" s="2"/>
       <c r="S76" s="2"/>
       <c r="T76" s="2"/>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" ht="14.25" customHeight="1">
       <c r="A77" s="2">
-        <v>46</v>
+        <v>46.0</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>20</v>
@@ -3933,18 +3825,10 @@
         <v>22</v>
       </c>
       <c r="J77" s="2"/>
-      <c r="K77" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L77" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M77" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N77" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="K77" s="2"/>
+      <c r="L77" s="2"/>
+      <c r="M77" s="2"/>
+      <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
       <c r="Q77" s="2"/>
@@ -3952,9 +3836,9 @@
       <c r="S77" s="2"/>
       <c r="T77" s="2"/>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="2">
-        <v>46</v>
+        <v>46.0</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>20</v>
@@ -3962,12 +3846,24 @@
       <c r="C78" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="2"/>
-      <c r="I78" s="2"/>
+      <c r="D78" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
       <c r="L78" s="2"/>
@@ -3980,9 +3876,9 @@
       <c r="S78" s="2"/>
       <c r="T78" s="2"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="2">
-        <v>46</v>
+        <v>46.0</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>20</v>
@@ -4008,9 +3904,9 @@
       <c r="S79" s="2"/>
       <c r="T79" s="2"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" ht="14.25" customHeight="1">
       <c r="A80" s="2">
-        <v>113</v>
+        <v>113.0</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>28</v>
@@ -4036,9 +3932,9 @@
       <c r="S80" s="2"/>
       <c r="T80" s="2"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="2">
-        <v>113</v>
+        <v>113.0</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>28</v>
@@ -4064,9 +3960,9 @@
       <c r="S81" s="2"/>
       <c r="T81" s="2"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="2">
-        <v>113</v>
+        <v>113.0</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>28</v>
@@ -4092,9 +3988,9 @@
       <c r="S82" s="2"/>
       <c r="T82" s="2"/>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="83" ht="14.25" customHeight="1">
       <c r="A83" s="2">
-        <v>113</v>
+        <v>113.0</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>28</v>
@@ -4120,9 +4016,9 @@
       <c r="S83" s="2"/>
       <c r="T83" s="2"/>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="2">
-        <v>113</v>
+        <v>113.0</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>28</v>
@@ -4148,9 +4044,9 @@
       <c r="S84" s="2"/>
       <c r="T84" s="2"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="2">
-        <v>113</v>
+        <v>113.0</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>28</v>
@@ -4176,7 +4072,7 @@
       <c r="S85" s="2"/>
       <c r="T85" s="2"/>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" ht="14.25" customHeight="1">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4198,7 +4094,7 @@
       <c r="S86" s="2"/>
       <c r="T86" s="2"/>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4220,7 +4116,7 @@
       <c r="S87" s="2"/>
       <c r="T87" s="2"/>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -4242,7 +4138,7 @@
       <c r="S88" s="2"/>
       <c r="T88" s="2"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" ht="14.25" customHeight="1">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -4264,7 +4160,7 @@
       <c r="S89" s="2"/>
       <c r="T89" s="2"/>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -4286,7 +4182,7 @@
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -4308,7 +4204,7 @@
       <c r="S91" s="2"/>
       <c r="T91" s="2"/>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" ht="14.25" customHeight="1">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -4330,7 +4226,7 @@
       <c r="S92" s="2"/>
       <c r="T92" s="2"/>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -4352,7 +4248,7 @@
       <c r="S93" s="2"/>
       <c r="T93" s="2"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -4374,7 +4270,7 @@
       <c r="S94" s="2"/>
       <c r="T94" s="2"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" ht="14.25" customHeight="1">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -4396,7 +4292,7 @@
       <c r="S95" s="2"/>
       <c r="T95" s="2"/>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -4418,7 +4314,7 @@
       <c r="S96" s="2"/>
       <c r="T96" s="2"/>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -4440,7 +4336,7 @@
       <c r="S97" s="2"/>
       <c r="T97" s="2"/>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="98" ht="14.25" customHeight="1">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -4462,7 +4358,7 @@
       <c r="S98" s="2"/>
       <c r="T98" s="2"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -4484,7 +4380,7 @@
       <c r="S99" s="2"/>
       <c r="T99" s="2"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -4506,7 +4402,7 @@
       <c r="S100" s="2"/>
       <c r="T100" s="2"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="101" ht="14.25" customHeight="1">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -4528,7 +4424,7 @@
       <c r="S101" s="2"/>
       <c r="T101" s="2"/>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -4550,7 +4446,7 @@
       <c r="S102" s="2"/>
       <c r="T102" s="2"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -4572,7 +4468,7 @@
       <c r="S103" s="2"/>
       <c r="T103" s="2"/>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="104" ht="14.25" customHeight="1">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -4594,7 +4490,7 @@
       <c r="S104" s="2"/>
       <c r="T104" s="2"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
@@ -4616,7 +4512,7 @@
       <c r="S105" s="2"/>
       <c r="T105" s="2"/>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -4638,7 +4534,7 @@
       <c r="S106" s="2"/>
       <c r="T106" s="2"/>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="107" ht="14.25" customHeight="1">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -4660,7 +4556,7 @@
       <c r="S107" s="2"/>
       <c r="T107" s="2"/>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
@@ -4682,7 +4578,7 @@
       <c r="S108" s="2"/>
       <c r="T108" s="2"/>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
@@ -4704,7 +4600,7 @@
       <c r="S109" s="2"/>
       <c r="T109" s="2"/>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" ht="14.25" customHeight="1">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
@@ -4726,7 +4622,7 @@
       <c r="S110" s="2"/>
       <c r="T110" s="2"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
@@ -4748,7 +4644,7 @@
       <c r="S111" s="2"/>
       <c r="T111" s="2"/>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
@@ -4770,7 +4666,7 @@
       <c r="S112" s="2"/>
       <c r="T112" s="2"/>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="113" ht="14.25" customHeight="1">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
@@ -4792,7 +4688,7 @@
       <c r="S113" s="2"/>
       <c r="T113" s="2"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
@@ -4814,7 +4710,7 @@
       <c r="S114" s="2"/>
       <c r="T114" s="2"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -4836,7 +4732,7 @@
       <c r="S115" s="2"/>
       <c r="T115" s="2"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="116" ht="14.25" customHeight="1">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -4858,7 +4754,7 @@
       <c r="S116" s="2"/>
       <c r="T116" s="2"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="117" ht="14.25" customHeight="1">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
@@ -4880,7 +4776,7 @@
       <c r="S117" s="2"/>
       <c r="T117" s="2"/>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="118" ht="14.25" customHeight="1">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
@@ -4902,7 +4798,7 @@
       <c r="S118" s="2"/>
       <c r="T118" s="2"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="119" ht="14.25" customHeight="1">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -4924,7 +4820,7 @@
       <c r="S119" s="2"/>
       <c r="T119" s="2"/>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="120" ht="14.25" customHeight="1">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
@@ -4946,7 +4842,7 @@
       <c r="S120" s="2"/>
       <c r="T120" s="2"/>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="121" ht="14.25" customHeight="1">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -4968,7 +4864,7 @@
       <c r="S121" s="2"/>
       <c r="T121" s="2"/>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="122" ht="14.25" customHeight="1">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
@@ -4990,7 +4886,7 @@
       <c r="S122" s="2"/>
       <c r="T122" s="2"/>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="123" ht="14.25" customHeight="1">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -5012,7 +4908,7 @@
       <c r="S123" s="2"/>
       <c r="T123" s="2"/>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="124" ht="14.25" customHeight="1">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
@@ -5034,7 +4930,7 @@
       <c r="S124" s="2"/>
       <c r="T124" s="2"/>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="125" ht="14.25" customHeight="1">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -5056,7 +4952,7 @@
       <c r="S125" s="2"/>
       <c r="T125" s="2"/>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="126" ht="14.25" customHeight="1">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -5078,7 +4974,7 @@
       <c r="S126" s="2"/>
       <c r="T126" s="2"/>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="127" ht="14.25" customHeight="1">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -5100,7 +4996,7 @@
       <c r="S127" s="2"/>
       <c r="T127" s="2"/>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="128" ht="14.25" customHeight="1">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
@@ -5122,7 +5018,7 @@
       <c r="S128" s="2"/>
       <c r="T128" s="2"/>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="129" ht="14.25" customHeight="1">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -5144,7 +5040,7 @@
       <c r="S129" s="2"/>
       <c r="T129" s="2"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="130" ht="14.25" customHeight="1">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -5166,7 +5062,7 @@
       <c r="S130" s="2"/>
       <c r="T130" s="2"/>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="131" ht="14.25" customHeight="1">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -5188,7 +5084,7 @@
       <c r="S131" s="2"/>
       <c r="T131" s="2"/>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="132" ht="14.25" customHeight="1">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -5210,7 +5106,7 @@
       <c r="S132" s="2"/>
       <c r="T132" s="2"/>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="133" ht="14.25" customHeight="1">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -5232,7 +5128,7 @@
       <c r="S133" s="2"/>
       <c r="T133" s="2"/>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="134" ht="14.25" customHeight="1">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -5254,7 +5150,7 @@
       <c r="S134" s="2"/>
       <c r="T134" s="2"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="135" ht="14.25" customHeight="1">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -5276,7 +5172,7 @@
       <c r="S135" s="2"/>
       <c r="T135" s="2"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="136" ht="14.25" customHeight="1">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -5298,7 +5194,7 @@
       <c r="S136" s="2"/>
       <c r="T136" s="2"/>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="137" ht="14.25" customHeight="1">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -5320,7 +5216,7 @@
       <c r="S137" s="2"/>
       <c r="T137" s="2"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="138" ht="14.25" customHeight="1">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -5342,7 +5238,7 @@
       <c r="S138" s="2"/>
       <c r="T138" s="2"/>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="139" ht="14.25" customHeight="1">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
@@ -5364,7 +5260,7 @@
       <c r="S139" s="2"/>
       <c r="T139" s="2"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="140" ht="14.25" customHeight="1">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
@@ -5386,7 +5282,7 @@
       <c r="S140" s="2"/>
       <c r="T140" s="2"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="141" ht="14.25" customHeight="1">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
@@ -5408,7 +5304,7 @@
       <c r="S141" s="2"/>
       <c r="T141" s="2"/>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="142" ht="14.25" customHeight="1">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
@@ -5430,7 +5326,7 @@
       <c r="S142" s="2"/>
       <c r="T142" s="2"/>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="143" ht="14.25" customHeight="1">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -5452,7 +5348,7 @@
       <c r="S143" s="2"/>
       <c r="T143" s="2"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="144" ht="14.25" customHeight="1">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
@@ -5474,7 +5370,7 @@
       <c r="S144" s="2"/>
       <c r="T144" s="2"/>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="145" ht="14.25" customHeight="1">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -5496,7 +5392,7 @@
       <c r="S145" s="2"/>
       <c r="T145" s="2"/>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="146" ht="14.25" customHeight="1">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
@@ -5518,7 +5414,7 @@
       <c r="S146" s="2"/>
       <c r="T146" s="2"/>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="147" ht="14.25" customHeight="1">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -5540,7 +5436,7 @@
       <c r="S147" s="2"/>
       <c r="T147" s="2"/>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="148" ht="14.25" customHeight="1">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
@@ -5562,7 +5458,7 @@
       <c r="S148" s="2"/>
       <c r="T148" s="2"/>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="149" ht="14.25" customHeight="1">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -5584,7 +5480,7 @@
       <c r="S149" s="2"/>
       <c r="T149" s="2"/>
     </row>
-    <row r="150" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="150" ht="14.25" customHeight="1">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
@@ -5606,7 +5502,7 @@
       <c r="S150" s="2"/>
       <c r="T150" s="2"/>
     </row>
-    <row r="151" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="151" ht="14.25" customHeight="1">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -5628,7 +5524,7 @@
       <c r="S151" s="2"/>
       <c r="T151" s="2"/>
     </row>
-    <row r="152" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="152" ht="14.25" customHeight="1">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
@@ -5650,7 +5546,7 @@
       <c r="S152" s="2"/>
       <c r="T152" s="2"/>
     </row>
-    <row r="153" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="153" ht="14.25" customHeight="1">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -5672,7 +5568,7 @@
       <c r="S153" s="2"/>
       <c r="T153" s="2"/>
     </row>
-    <row r="154" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="154" ht="14.25" customHeight="1">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
@@ -5694,7 +5590,7 @@
       <c r="S154" s="2"/>
       <c r="T154" s="2"/>
     </row>
-    <row r="155" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="155" ht="14.25" customHeight="1">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
@@ -5716,7 +5612,7 @@
       <c r="S155" s="2"/>
       <c r="T155" s="2"/>
     </row>
-    <row r="156" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="156" ht="14.25" customHeight="1">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
@@ -5738,7 +5634,7 @@
       <c r="S156" s="2"/>
       <c r="T156" s="2"/>
     </row>
-    <row r="157" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="157" ht="14.25" customHeight="1">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
@@ -5760,7 +5656,7 @@
       <c r="S157" s="2"/>
       <c r="T157" s="2"/>
     </row>
-    <row r="158" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="158" ht="14.25" customHeight="1">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
@@ -5782,7 +5678,7 @@
       <c r="S158" s="2"/>
       <c r="T158" s="2"/>
     </row>
-    <row r="159" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="159" ht="14.25" customHeight="1">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
@@ -5804,7 +5700,7 @@
       <c r="S159" s="2"/>
       <c r="T159" s="2"/>
     </row>
-    <row r="160" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="160" ht="14.25" customHeight="1">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
@@ -5826,7 +5722,7 @@
       <c r="S160" s="2"/>
       <c r="T160" s="2"/>
     </row>
-    <row r="161" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="161" ht="14.25" customHeight="1">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
@@ -5848,7 +5744,7 @@
       <c r="S161" s="2"/>
       <c r="T161" s="2"/>
     </row>
-    <row r="162" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="162" ht="14.25" customHeight="1">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
@@ -5870,7 +5766,7 @@
       <c r="S162" s="2"/>
       <c r="T162" s="2"/>
     </row>
-    <row r="163" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="163" ht="14.25" customHeight="1">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
@@ -5892,7 +5788,7 @@
       <c r="S163" s="2"/>
       <c r="T163" s="2"/>
     </row>
-    <row r="164" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="164" ht="14.25" customHeight="1">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
@@ -5914,7 +5810,7 @@
       <c r="S164" s="2"/>
       <c r="T164" s="2"/>
     </row>
-    <row r="165" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="165" ht="14.25" customHeight="1">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
@@ -5936,7 +5832,7 @@
       <c r="S165" s="2"/>
       <c r="T165" s="2"/>
     </row>
-    <row r="166" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="166" ht="14.25" customHeight="1">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
@@ -5958,7 +5854,7 @@
       <c r="S166" s="2"/>
       <c r="T166" s="2"/>
     </row>
-    <row r="167" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="167" ht="14.25" customHeight="1">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -5980,7 +5876,7 @@
       <c r="S167" s="2"/>
       <c r="T167" s="2"/>
     </row>
-    <row r="168" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="168" ht="14.25" customHeight="1">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
@@ -6002,7 +5898,7 @@
       <c r="S168" s="2"/>
       <c r="T168" s="2"/>
     </row>
-    <row r="169" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="169" ht="14.25" customHeight="1">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -6024,7 +5920,7 @@
       <c r="S169" s="2"/>
       <c r="T169" s="2"/>
     </row>
-    <row r="170" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="170" ht="14.25" customHeight="1">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
@@ -6046,7 +5942,7 @@
       <c r="S170" s="2"/>
       <c r="T170" s="2"/>
     </row>
-    <row r="171" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="171" ht="14.25" customHeight="1">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -6068,7 +5964,7 @@
       <c r="S171" s="2"/>
       <c r="T171" s="2"/>
     </row>
-    <row r="172" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="172" ht="14.25" customHeight="1">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
@@ -6090,7 +5986,7 @@
       <c r="S172" s="2"/>
       <c r="T172" s="2"/>
     </row>
-    <row r="173" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="173" ht="14.25" customHeight="1">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
@@ -6112,7 +6008,7 @@
       <c r="S173" s="2"/>
       <c r="T173" s="2"/>
     </row>
-    <row r="174" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="174" ht="14.25" customHeight="1">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
@@ -6134,7 +6030,7 @@
       <c r="S174" s="2"/>
       <c r="T174" s="2"/>
     </row>
-    <row r="175" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="175" ht="14.25" customHeight="1">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
@@ -6156,7 +6052,7 @@
       <c r="S175" s="2"/>
       <c r="T175" s="2"/>
     </row>
-    <row r="176" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="176" ht="14.25" customHeight="1">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
@@ -6178,7 +6074,7 @@
       <c r="S176" s="2"/>
       <c r="T176" s="2"/>
     </row>
-    <row r="177" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="177" ht="14.25" customHeight="1">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
@@ -6200,7 +6096,7 @@
       <c r="S177" s="2"/>
       <c r="T177" s="2"/>
     </row>
-    <row r="178" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="178" ht="14.25" customHeight="1">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
@@ -6222,7 +6118,7 @@
       <c r="S178" s="2"/>
       <c r="T178" s="2"/>
     </row>
-    <row r="179" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="179" ht="14.25" customHeight="1">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
@@ -6244,7 +6140,7 @@
       <c r="S179" s="2"/>
       <c r="T179" s="2"/>
     </row>
-    <row r="180" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="180" ht="14.25" customHeight="1">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
@@ -6266,7 +6162,7 @@
       <c r="S180" s="2"/>
       <c r="T180" s="2"/>
     </row>
-    <row r="181" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="181" ht="14.25" customHeight="1">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
@@ -6288,7 +6184,7 @@
       <c r="S181" s="2"/>
       <c r="T181" s="2"/>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="182" ht="14.25" customHeight="1">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
@@ -6310,7 +6206,7 @@
       <c r="S182" s="2"/>
       <c r="T182" s="2"/>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="183" ht="14.25" customHeight="1">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
@@ -6332,7 +6228,7 @@
       <c r="S183" s="2"/>
       <c r="T183" s="2"/>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="184" ht="14.25" customHeight="1">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
@@ -6354,7 +6250,7 @@
       <c r="S184" s="2"/>
       <c r="T184" s="2"/>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="185" ht="14.25" customHeight="1">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
@@ -6376,7 +6272,7 @@
       <c r="S185" s="2"/>
       <c r="T185" s="2"/>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="186" ht="14.25" customHeight="1">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
       <c r="C186" s="2"/>
@@ -6398,7 +6294,7 @@
       <c r="S186" s="2"/>
       <c r="T186" s="2"/>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="187" ht="14.25" customHeight="1">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
@@ -6420,7 +6316,7 @@
       <c r="S187" s="2"/>
       <c r="T187" s="2"/>
     </row>
-    <row r="188" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="188" ht="14.25" customHeight="1">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
       <c r="C188" s="2"/>
@@ -6442,7 +6338,7 @@
       <c r="S188" s="2"/>
       <c r="T188" s="2"/>
     </row>
-    <row r="189" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="189" ht="14.25" customHeight="1">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -6464,7 +6360,7 @@
       <c r="S189" s="2"/>
       <c r="T189" s="2"/>
     </row>
-    <row r="190" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="190" ht="14.25" customHeight="1">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="2"/>
@@ -6486,7 +6382,7 @@
       <c r="S190" s="2"/>
       <c r="T190" s="2"/>
     </row>
-    <row r="191" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="191" ht="14.25" customHeight="1">
       <c r="E191" s="2"/>
       <c r="F191" s="2"/>
       <c r="G191" s="2"/>
@@ -6504,7 +6400,7 @@
       <c r="S191" s="2"/>
       <c r="T191" s="2"/>
     </row>
-    <row r="192" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="192" ht="14.25" customHeight="1">
       <c r="E192" s="2"/>
       <c r="F192" s="2"/>
       <c r="G192" s="2"/>
@@ -6522,7 +6418,7 @@
       <c r="S192" s="2"/>
       <c r="T192" s="2"/>
     </row>
-    <row r="193" spans="5:20" x14ac:dyDescent="0.3">
+    <row r="193" ht="14.25" customHeight="1">
       <c r="E193" s="2"/>
       <c r="F193" s="2"/>
       <c r="G193" s="2"/>
@@ -6540,7 +6436,7 @@
       <c r="S193" s="2"/>
       <c r="T193" s="2"/>
     </row>
-    <row r="194" spans="5:20" x14ac:dyDescent="0.3">
+    <row r="194" ht="14.25" customHeight="1">
       <c r="E194" s="2"/>
       <c r="F194" s="2"/>
       <c r="G194" s="2"/>
@@ -6558,7 +6454,7 @@
       <c r="S194" s="2"/>
       <c r="T194" s="2"/>
     </row>
-    <row r="195" spans="5:20" x14ac:dyDescent="0.3">
+    <row r="195" ht="14.25" customHeight="1">
       <c r="E195" s="2"/>
       <c r="F195" s="2"/>
       <c r="G195" s="2"/>
@@ -6576,7 +6472,7 @@
       <c r="S195" s="2"/>
       <c r="T195" s="2"/>
     </row>
-    <row r="196" spans="5:20" x14ac:dyDescent="0.3">
+    <row r="196" ht="14.25" customHeight="1">
       <c r="E196" s="2"/>
       <c r="F196" s="2"/>
       <c r="G196" s="2"/>
@@ -6594,8 +6490,814 @@
       <c r="S196" s="2"/>
       <c r="T196" s="2"/>
     </row>
+    <row r="197" ht="14.25" customHeight="1"/>
+    <row r="198" ht="14.25" customHeight="1"/>
+    <row r="199" ht="14.25" customHeight="1"/>
+    <row r="200" ht="14.25" customHeight="1"/>
+    <row r="201" ht="14.25" customHeight="1"/>
+    <row r="202" ht="14.25" customHeight="1"/>
+    <row r="203" ht="14.25" customHeight="1"/>
+    <row r="204" ht="14.25" customHeight="1"/>
+    <row r="205" ht="14.25" customHeight="1"/>
+    <row r="206" ht="14.25" customHeight="1"/>
+    <row r="207" ht="14.25" customHeight="1"/>
+    <row r="208" ht="14.25" customHeight="1"/>
+    <row r="209" ht="14.25" customHeight="1"/>
+    <row r="210" ht="14.25" customHeight="1"/>
+    <row r="211" ht="14.25" customHeight="1"/>
+    <row r="212" ht="14.25" customHeight="1"/>
+    <row r="213" ht="14.25" customHeight="1"/>
+    <row r="214" ht="14.25" customHeight="1"/>
+    <row r="215" ht="14.25" customHeight="1"/>
+    <row r="216" ht="14.25" customHeight="1"/>
+    <row r="217" ht="14.25" customHeight="1"/>
+    <row r="218" ht="14.25" customHeight="1"/>
+    <row r="219" ht="14.25" customHeight="1"/>
+    <row r="220" ht="14.25" customHeight="1"/>
+    <row r="221" ht="14.25" customHeight="1"/>
+    <row r="222" ht="14.25" customHeight="1"/>
+    <row r="223" ht="14.25" customHeight="1"/>
+    <row r="224" ht="14.25" customHeight="1"/>
+    <row r="225" ht="14.25" customHeight="1"/>
+    <row r="226" ht="14.25" customHeight="1"/>
+    <row r="227" ht="14.25" customHeight="1"/>
+    <row r="228" ht="14.25" customHeight="1"/>
+    <row r="229" ht="14.25" customHeight="1"/>
+    <row r="230" ht="14.25" customHeight="1"/>
+    <row r="231" ht="14.25" customHeight="1"/>
+    <row r="232" ht="14.25" customHeight="1"/>
+    <row r="233" ht="14.25" customHeight="1"/>
+    <row r="234" ht="14.25" customHeight="1"/>
+    <row r="235" ht="14.25" customHeight="1"/>
+    <row r="236" ht="14.25" customHeight="1"/>
+    <row r="237" ht="14.25" customHeight="1"/>
+    <row r="238" ht="14.25" customHeight="1"/>
+    <row r="239" ht="14.25" customHeight="1"/>
+    <row r="240" ht="14.25" customHeight="1"/>
+    <row r="241" ht="14.25" customHeight="1"/>
+    <row r="242" ht="14.25" customHeight="1"/>
+    <row r="243" ht="14.25" customHeight="1"/>
+    <row r="244" ht="14.25" customHeight="1"/>
+    <row r="245" ht="14.25" customHeight="1"/>
+    <row r="246" ht="14.25" customHeight="1"/>
+    <row r="247" ht="14.25" customHeight="1"/>
+    <row r="248" ht="14.25" customHeight="1"/>
+    <row r="249" ht="14.25" customHeight="1"/>
+    <row r="250" ht="14.25" customHeight="1"/>
+    <row r="251" ht="14.25" customHeight="1"/>
+    <row r="252" ht="14.25" customHeight="1"/>
+    <row r="253" ht="14.25" customHeight="1"/>
+    <row r="254" ht="14.25" customHeight="1"/>
+    <row r="255" ht="14.25" customHeight="1"/>
+    <row r="256" ht="14.25" customHeight="1"/>
+    <row r="257" ht="14.25" customHeight="1"/>
+    <row r="258" ht="14.25" customHeight="1"/>
+    <row r="259" ht="14.25" customHeight="1"/>
+    <row r="260" ht="14.25" customHeight="1"/>
+    <row r="261" ht="14.25" customHeight="1"/>
+    <row r="262" ht="14.25" customHeight="1"/>
+    <row r="263" ht="14.25" customHeight="1"/>
+    <row r="264" ht="14.25" customHeight="1"/>
+    <row r="265" ht="14.25" customHeight="1"/>
+    <row r="266" ht="14.25" customHeight="1"/>
+    <row r="267" ht="14.25" customHeight="1"/>
+    <row r="268" ht="14.25" customHeight="1"/>
+    <row r="269" ht="14.25" customHeight="1"/>
+    <row r="270" ht="14.25" customHeight="1"/>
+    <row r="271" ht="14.25" customHeight="1"/>
+    <row r="272" ht="14.25" customHeight="1"/>
+    <row r="273" ht="14.25" customHeight="1"/>
+    <row r="274" ht="14.25" customHeight="1"/>
+    <row r="275" ht="14.25" customHeight="1"/>
+    <row r="276" ht="14.25" customHeight="1"/>
+    <row r="277" ht="14.25" customHeight="1"/>
+    <row r="278" ht="14.25" customHeight="1"/>
+    <row r="279" ht="14.25" customHeight="1"/>
+    <row r="280" ht="14.25" customHeight="1"/>
+    <row r="281" ht="14.25" customHeight="1"/>
+    <row r="282" ht="14.25" customHeight="1"/>
+    <row r="283" ht="14.25" customHeight="1"/>
+    <row r="284" ht="14.25" customHeight="1"/>
+    <row r="285" ht="14.25" customHeight="1"/>
+    <row r="286" ht="14.25" customHeight="1"/>
+    <row r="287" ht="14.25" customHeight="1"/>
+    <row r="288" ht="14.25" customHeight="1"/>
+    <row r="289" ht="14.25" customHeight="1"/>
+    <row r="290" ht="14.25" customHeight="1"/>
+    <row r="291" ht="14.25" customHeight="1"/>
+    <row r="292" ht="14.25" customHeight="1"/>
+    <row r="293" ht="14.25" customHeight="1"/>
+    <row r="294" ht="14.25" customHeight="1"/>
+    <row r="295" ht="14.25" customHeight="1"/>
+    <row r="296" ht="14.25" customHeight="1"/>
+    <row r="297" ht="14.25" customHeight="1"/>
+    <row r="298" ht="14.25" customHeight="1"/>
+    <row r="299" ht="14.25" customHeight="1"/>
+    <row r="300" ht="14.25" customHeight="1"/>
+    <row r="301" ht="14.25" customHeight="1"/>
+    <row r="302" ht="14.25" customHeight="1"/>
+    <row r="303" ht="14.25" customHeight="1"/>
+    <row r="304" ht="14.25" customHeight="1"/>
+    <row r="305" ht="14.25" customHeight="1"/>
+    <row r="306" ht="14.25" customHeight="1"/>
+    <row r="307" ht="14.25" customHeight="1"/>
+    <row r="308" ht="14.25" customHeight="1"/>
+    <row r="309" ht="14.25" customHeight="1"/>
+    <row r="310" ht="14.25" customHeight="1"/>
+    <row r="311" ht="14.25" customHeight="1"/>
+    <row r="312" ht="14.25" customHeight="1"/>
+    <row r="313" ht="14.25" customHeight="1"/>
+    <row r="314" ht="14.25" customHeight="1"/>
+    <row r="315" ht="14.25" customHeight="1"/>
+    <row r="316" ht="14.25" customHeight="1"/>
+    <row r="317" ht="14.25" customHeight="1"/>
+    <row r="318" ht="14.25" customHeight="1"/>
+    <row r="319" ht="14.25" customHeight="1"/>
+    <row r="320" ht="14.25" customHeight="1"/>
+    <row r="321" ht="14.25" customHeight="1"/>
+    <row r="322" ht="14.25" customHeight="1"/>
+    <row r="323" ht="14.25" customHeight="1"/>
+    <row r="324" ht="14.25" customHeight="1"/>
+    <row r="325" ht="14.25" customHeight="1"/>
+    <row r="326" ht="14.25" customHeight="1"/>
+    <row r="327" ht="14.25" customHeight="1"/>
+    <row r="328" ht="14.25" customHeight="1"/>
+    <row r="329" ht="14.25" customHeight="1"/>
+    <row r="330" ht="14.25" customHeight="1"/>
+    <row r="331" ht="14.25" customHeight="1"/>
+    <row r="332" ht="14.25" customHeight="1"/>
+    <row r="333" ht="14.25" customHeight="1"/>
+    <row r="334" ht="14.25" customHeight="1"/>
+    <row r="335" ht="14.25" customHeight="1"/>
+    <row r="336" ht="14.25" customHeight="1"/>
+    <row r="337" ht="14.25" customHeight="1"/>
+    <row r="338" ht="14.25" customHeight="1"/>
+    <row r="339" ht="14.25" customHeight="1"/>
+    <row r="340" ht="14.25" customHeight="1"/>
+    <row r="341" ht="14.25" customHeight="1"/>
+    <row r="342" ht="14.25" customHeight="1"/>
+    <row r="343" ht="14.25" customHeight="1"/>
+    <row r="344" ht="14.25" customHeight="1"/>
+    <row r="345" ht="14.25" customHeight="1"/>
+    <row r="346" ht="14.25" customHeight="1"/>
+    <row r="347" ht="14.25" customHeight="1"/>
+    <row r="348" ht="14.25" customHeight="1"/>
+    <row r="349" ht="14.25" customHeight="1"/>
+    <row r="350" ht="14.25" customHeight="1"/>
+    <row r="351" ht="14.25" customHeight="1"/>
+    <row r="352" ht="14.25" customHeight="1"/>
+    <row r="353" ht="14.25" customHeight="1"/>
+    <row r="354" ht="14.25" customHeight="1"/>
+    <row r="355" ht="14.25" customHeight="1"/>
+    <row r="356" ht="14.25" customHeight="1"/>
+    <row r="357" ht="14.25" customHeight="1"/>
+    <row r="358" ht="14.25" customHeight="1"/>
+    <row r="359" ht="14.25" customHeight="1"/>
+    <row r="360" ht="14.25" customHeight="1"/>
+    <row r="361" ht="14.25" customHeight="1"/>
+    <row r="362" ht="14.25" customHeight="1"/>
+    <row r="363" ht="14.25" customHeight="1"/>
+    <row r="364" ht="14.25" customHeight="1"/>
+    <row r="365" ht="14.25" customHeight="1"/>
+    <row r="366" ht="14.25" customHeight="1"/>
+    <row r="367" ht="14.25" customHeight="1"/>
+    <row r="368" ht="14.25" customHeight="1"/>
+    <row r="369" ht="14.25" customHeight="1"/>
+    <row r="370" ht="14.25" customHeight="1"/>
+    <row r="371" ht="14.25" customHeight="1"/>
+    <row r="372" ht="14.25" customHeight="1"/>
+    <row r="373" ht="14.25" customHeight="1"/>
+    <row r="374" ht="14.25" customHeight="1"/>
+    <row r="375" ht="14.25" customHeight="1"/>
+    <row r="376" ht="14.25" customHeight="1"/>
+    <row r="377" ht="14.25" customHeight="1"/>
+    <row r="378" ht="14.25" customHeight="1"/>
+    <row r="379" ht="14.25" customHeight="1"/>
+    <row r="380" ht="14.25" customHeight="1"/>
+    <row r="381" ht="14.25" customHeight="1"/>
+    <row r="382" ht="14.25" customHeight="1"/>
+    <row r="383" ht="14.25" customHeight="1"/>
+    <row r="384" ht="14.25" customHeight="1"/>
+    <row r="385" ht="14.25" customHeight="1"/>
+    <row r="386" ht="14.25" customHeight="1"/>
+    <row r="387" ht="14.25" customHeight="1"/>
+    <row r="388" ht="14.25" customHeight="1"/>
+    <row r="389" ht="14.25" customHeight="1"/>
+    <row r="390" ht="14.25" customHeight="1"/>
+    <row r="391" ht="14.25" customHeight="1"/>
+    <row r="392" ht="14.25" customHeight="1"/>
+    <row r="393" ht="14.25" customHeight="1"/>
+    <row r="394" ht="14.25" customHeight="1"/>
+    <row r="395" ht="14.25" customHeight="1"/>
+    <row r="396" ht="14.25" customHeight="1"/>
+    <row r="397" ht="14.25" customHeight="1"/>
+    <row r="398" ht="14.25" customHeight="1"/>
+    <row r="399" ht="14.25" customHeight="1"/>
+    <row r="400" ht="14.25" customHeight="1"/>
+    <row r="401" ht="14.25" customHeight="1"/>
+    <row r="402" ht="14.25" customHeight="1"/>
+    <row r="403" ht="14.25" customHeight="1"/>
+    <row r="404" ht="14.25" customHeight="1"/>
+    <row r="405" ht="14.25" customHeight="1"/>
+    <row r="406" ht="14.25" customHeight="1"/>
+    <row r="407" ht="14.25" customHeight="1"/>
+    <row r="408" ht="14.25" customHeight="1"/>
+    <row r="409" ht="14.25" customHeight="1"/>
+    <row r="410" ht="14.25" customHeight="1"/>
+    <row r="411" ht="14.25" customHeight="1"/>
+    <row r="412" ht="14.25" customHeight="1"/>
+    <row r="413" ht="14.25" customHeight="1"/>
+    <row r="414" ht="14.25" customHeight="1"/>
+    <row r="415" ht="14.25" customHeight="1"/>
+    <row r="416" ht="14.25" customHeight="1"/>
+    <row r="417" ht="14.25" customHeight="1"/>
+    <row r="418" ht="14.25" customHeight="1"/>
+    <row r="419" ht="14.25" customHeight="1"/>
+    <row r="420" ht="14.25" customHeight="1"/>
+    <row r="421" ht="14.25" customHeight="1"/>
+    <row r="422" ht="14.25" customHeight="1"/>
+    <row r="423" ht="14.25" customHeight="1"/>
+    <row r="424" ht="14.25" customHeight="1"/>
+    <row r="425" ht="14.25" customHeight="1"/>
+    <row r="426" ht="14.25" customHeight="1"/>
+    <row r="427" ht="14.25" customHeight="1"/>
+    <row r="428" ht="14.25" customHeight="1"/>
+    <row r="429" ht="14.25" customHeight="1"/>
+    <row r="430" ht="14.25" customHeight="1"/>
+    <row r="431" ht="14.25" customHeight="1"/>
+    <row r="432" ht="14.25" customHeight="1"/>
+    <row r="433" ht="14.25" customHeight="1"/>
+    <row r="434" ht="14.25" customHeight="1"/>
+    <row r="435" ht="14.25" customHeight="1"/>
+    <row r="436" ht="14.25" customHeight="1"/>
+    <row r="437" ht="14.25" customHeight="1"/>
+    <row r="438" ht="14.25" customHeight="1"/>
+    <row r="439" ht="14.25" customHeight="1"/>
+    <row r="440" ht="14.25" customHeight="1"/>
+    <row r="441" ht="14.25" customHeight="1"/>
+    <row r="442" ht="14.25" customHeight="1"/>
+    <row r="443" ht="14.25" customHeight="1"/>
+    <row r="444" ht="14.25" customHeight="1"/>
+    <row r="445" ht="14.25" customHeight="1"/>
+    <row r="446" ht="14.25" customHeight="1"/>
+    <row r="447" ht="14.25" customHeight="1"/>
+    <row r="448" ht="14.25" customHeight="1"/>
+    <row r="449" ht="14.25" customHeight="1"/>
+    <row r="450" ht="14.25" customHeight="1"/>
+    <row r="451" ht="14.25" customHeight="1"/>
+    <row r="452" ht="14.25" customHeight="1"/>
+    <row r="453" ht="14.25" customHeight="1"/>
+    <row r="454" ht="14.25" customHeight="1"/>
+    <row r="455" ht="14.25" customHeight="1"/>
+    <row r="456" ht="14.25" customHeight="1"/>
+    <row r="457" ht="14.25" customHeight="1"/>
+    <row r="458" ht="14.25" customHeight="1"/>
+    <row r="459" ht="14.25" customHeight="1"/>
+    <row r="460" ht="14.25" customHeight="1"/>
+    <row r="461" ht="14.25" customHeight="1"/>
+    <row r="462" ht="14.25" customHeight="1"/>
+    <row r="463" ht="14.25" customHeight="1"/>
+    <row r="464" ht="14.25" customHeight="1"/>
+    <row r="465" ht="14.25" customHeight="1"/>
+    <row r="466" ht="14.25" customHeight="1"/>
+    <row r="467" ht="14.25" customHeight="1"/>
+    <row r="468" ht="14.25" customHeight="1"/>
+    <row r="469" ht="14.25" customHeight="1"/>
+    <row r="470" ht="14.25" customHeight="1"/>
+    <row r="471" ht="14.25" customHeight="1"/>
+    <row r="472" ht="14.25" customHeight="1"/>
+    <row r="473" ht="14.25" customHeight="1"/>
+    <row r="474" ht="14.25" customHeight="1"/>
+    <row r="475" ht="14.25" customHeight="1"/>
+    <row r="476" ht="14.25" customHeight="1"/>
+    <row r="477" ht="14.25" customHeight="1"/>
+    <row r="478" ht="14.25" customHeight="1"/>
+    <row r="479" ht="14.25" customHeight="1"/>
+    <row r="480" ht="14.25" customHeight="1"/>
+    <row r="481" ht="14.25" customHeight="1"/>
+    <row r="482" ht="14.25" customHeight="1"/>
+    <row r="483" ht="14.25" customHeight="1"/>
+    <row r="484" ht="14.25" customHeight="1"/>
+    <row r="485" ht="14.25" customHeight="1"/>
+    <row r="486" ht="14.25" customHeight="1"/>
+    <row r="487" ht="14.25" customHeight="1"/>
+    <row r="488" ht="14.25" customHeight="1"/>
+    <row r="489" ht="14.25" customHeight="1"/>
+    <row r="490" ht="14.25" customHeight="1"/>
+    <row r="491" ht="14.25" customHeight="1"/>
+    <row r="492" ht="14.25" customHeight="1"/>
+    <row r="493" ht="14.25" customHeight="1"/>
+    <row r="494" ht="14.25" customHeight="1"/>
+    <row r="495" ht="14.25" customHeight="1"/>
+    <row r="496" ht="14.25" customHeight="1"/>
+    <row r="497" ht="14.25" customHeight="1"/>
+    <row r="498" ht="14.25" customHeight="1"/>
+    <row r="499" ht="14.25" customHeight="1"/>
+    <row r="500" ht="14.25" customHeight="1"/>
+    <row r="501" ht="14.25" customHeight="1"/>
+    <row r="502" ht="14.25" customHeight="1"/>
+    <row r="503" ht="14.25" customHeight="1"/>
+    <row r="504" ht="14.25" customHeight="1"/>
+    <row r="505" ht="14.25" customHeight="1"/>
+    <row r="506" ht="14.25" customHeight="1"/>
+    <row r="507" ht="14.25" customHeight="1"/>
+    <row r="508" ht="14.25" customHeight="1"/>
+    <row r="509" ht="14.25" customHeight="1"/>
+    <row r="510" ht="14.25" customHeight="1"/>
+    <row r="511" ht="14.25" customHeight="1"/>
+    <row r="512" ht="14.25" customHeight="1"/>
+    <row r="513" ht="14.25" customHeight="1"/>
+    <row r="514" ht="14.25" customHeight="1"/>
+    <row r="515" ht="14.25" customHeight="1"/>
+    <row r="516" ht="14.25" customHeight="1"/>
+    <row r="517" ht="14.25" customHeight="1"/>
+    <row r="518" ht="14.25" customHeight="1"/>
+    <row r="519" ht="14.25" customHeight="1"/>
+    <row r="520" ht="14.25" customHeight="1"/>
+    <row r="521" ht="14.25" customHeight="1"/>
+    <row r="522" ht="14.25" customHeight="1"/>
+    <row r="523" ht="14.25" customHeight="1"/>
+    <row r="524" ht="14.25" customHeight="1"/>
+    <row r="525" ht="14.25" customHeight="1"/>
+    <row r="526" ht="14.25" customHeight="1"/>
+    <row r="527" ht="14.25" customHeight="1"/>
+    <row r="528" ht="14.25" customHeight="1"/>
+    <row r="529" ht="14.25" customHeight="1"/>
+    <row r="530" ht="14.25" customHeight="1"/>
+    <row r="531" ht="14.25" customHeight="1"/>
+    <row r="532" ht="14.25" customHeight="1"/>
+    <row r="533" ht="14.25" customHeight="1"/>
+    <row r="534" ht="14.25" customHeight="1"/>
+    <row r="535" ht="14.25" customHeight="1"/>
+    <row r="536" ht="14.25" customHeight="1"/>
+    <row r="537" ht="14.25" customHeight="1"/>
+    <row r="538" ht="14.25" customHeight="1"/>
+    <row r="539" ht="14.25" customHeight="1"/>
+    <row r="540" ht="14.25" customHeight="1"/>
+    <row r="541" ht="14.25" customHeight="1"/>
+    <row r="542" ht="14.25" customHeight="1"/>
+    <row r="543" ht="14.25" customHeight="1"/>
+    <row r="544" ht="14.25" customHeight="1"/>
+    <row r="545" ht="14.25" customHeight="1"/>
+    <row r="546" ht="14.25" customHeight="1"/>
+    <row r="547" ht="14.25" customHeight="1"/>
+    <row r="548" ht="14.25" customHeight="1"/>
+    <row r="549" ht="14.25" customHeight="1"/>
+    <row r="550" ht="14.25" customHeight="1"/>
+    <row r="551" ht="14.25" customHeight="1"/>
+    <row r="552" ht="14.25" customHeight="1"/>
+    <row r="553" ht="14.25" customHeight="1"/>
+    <row r="554" ht="14.25" customHeight="1"/>
+    <row r="555" ht="14.25" customHeight="1"/>
+    <row r="556" ht="14.25" customHeight="1"/>
+    <row r="557" ht="14.25" customHeight="1"/>
+    <row r="558" ht="14.25" customHeight="1"/>
+    <row r="559" ht="14.25" customHeight="1"/>
+    <row r="560" ht="14.25" customHeight="1"/>
+    <row r="561" ht="14.25" customHeight="1"/>
+    <row r="562" ht="14.25" customHeight="1"/>
+    <row r="563" ht="14.25" customHeight="1"/>
+    <row r="564" ht="14.25" customHeight="1"/>
+    <row r="565" ht="14.25" customHeight="1"/>
+    <row r="566" ht="14.25" customHeight="1"/>
+    <row r="567" ht="14.25" customHeight="1"/>
+    <row r="568" ht="14.25" customHeight="1"/>
+    <row r="569" ht="14.25" customHeight="1"/>
+    <row r="570" ht="14.25" customHeight="1"/>
+    <row r="571" ht="14.25" customHeight="1"/>
+    <row r="572" ht="14.25" customHeight="1"/>
+    <row r="573" ht="14.25" customHeight="1"/>
+    <row r="574" ht="14.25" customHeight="1"/>
+    <row r="575" ht="14.25" customHeight="1"/>
+    <row r="576" ht="14.25" customHeight="1"/>
+    <row r="577" ht="14.25" customHeight="1"/>
+    <row r="578" ht="14.25" customHeight="1"/>
+    <row r="579" ht="14.25" customHeight="1"/>
+    <row r="580" ht="14.25" customHeight="1"/>
+    <row r="581" ht="14.25" customHeight="1"/>
+    <row r="582" ht="14.25" customHeight="1"/>
+    <row r="583" ht="14.25" customHeight="1"/>
+    <row r="584" ht="14.25" customHeight="1"/>
+    <row r="585" ht="14.25" customHeight="1"/>
+    <row r="586" ht="14.25" customHeight="1"/>
+    <row r="587" ht="14.25" customHeight="1"/>
+    <row r="588" ht="14.25" customHeight="1"/>
+    <row r="589" ht="14.25" customHeight="1"/>
+    <row r="590" ht="14.25" customHeight="1"/>
+    <row r="591" ht="14.25" customHeight="1"/>
+    <row r="592" ht="14.25" customHeight="1"/>
+    <row r="593" ht="14.25" customHeight="1"/>
+    <row r="594" ht="14.25" customHeight="1"/>
+    <row r="595" ht="14.25" customHeight="1"/>
+    <row r="596" ht="14.25" customHeight="1"/>
+    <row r="597" ht="14.25" customHeight="1"/>
+    <row r="598" ht="14.25" customHeight="1"/>
+    <row r="599" ht="14.25" customHeight="1"/>
+    <row r="600" ht="14.25" customHeight="1"/>
+    <row r="601" ht="14.25" customHeight="1"/>
+    <row r="602" ht="14.25" customHeight="1"/>
+    <row r="603" ht="14.25" customHeight="1"/>
+    <row r="604" ht="14.25" customHeight="1"/>
+    <row r="605" ht="14.25" customHeight="1"/>
+    <row r="606" ht="14.25" customHeight="1"/>
+    <row r="607" ht="14.25" customHeight="1"/>
+    <row r="608" ht="14.25" customHeight="1"/>
+    <row r="609" ht="14.25" customHeight="1"/>
+    <row r="610" ht="14.25" customHeight="1"/>
+    <row r="611" ht="14.25" customHeight="1"/>
+    <row r="612" ht="14.25" customHeight="1"/>
+    <row r="613" ht="14.25" customHeight="1"/>
+    <row r="614" ht="14.25" customHeight="1"/>
+    <row r="615" ht="14.25" customHeight="1"/>
+    <row r="616" ht="14.25" customHeight="1"/>
+    <row r="617" ht="14.25" customHeight="1"/>
+    <row r="618" ht="14.25" customHeight="1"/>
+    <row r="619" ht="14.25" customHeight="1"/>
+    <row r="620" ht="14.25" customHeight="1"/>
+    <row r="621" ht="14.25" customHeight="1"/>
+    <row r="622" ht="14.25" customHeight="1"/>
+    <row r="623" ht="14.25" customHeight="1"/>
+    <row r="624" ht="14.25" customHeight="1"/>
+    <row r="625" ht="14.25" customHeight="1"/>
+    <row r="626" ht="14.25" customHeight="1"/>
+    <row r="627" ht="14.25" customHeight="1"/>
+    <row r="628" ht="14.25" customHeight="1"/>
+    <row r="629" ht="14.25" customHeight="1"/>
+    <row r="630" ht="14.25" customHeight="1"/>
+    <row r="631" ht="14.25" customHeight="1"/>
+    <row r="632" ht="14.25" customHeight="1"/>
+    <row r="633" ht="14.25" customHeight="1"/>
+    <row r="634" ht="14.25" customHeight="1"/>
+    <row r="635" ht="14.25" customHeight="1"/>
+    <row r="636" ht="14.25" customHeight="1"/>
+    <row r="637" ht="14.25" customHeight="1"/>
+    <row r="638" ht="14.25" customHeight="1"/>
+    <row r="639" ht="14.25" customHeight="1"/>
+    <row r="640" ht="14.25" customHeight="1"/>
+    <row r="641" ht="14.25" customHeight="1"/>
+    <row r="642" ht="14.25" customHeight="1"/>
+    <row r="643" ht="14.25" customHeight="1"/>
+    <row r="644" ht="14.25" customHeight="1"/>
+    <row r="645" ht="14.25" customHeight="1"/>
+    <row r="646" ht="14.25" customHeight="1"/>
+    <row r="647" ht="14.25" customHeight="1"/>
+    <row r="648" ht="14.25" customHeight="1"/>
+    <row r="649" ht="14.25" customHeight="1"/>
+    <row r="650" ht="14.25" customHeight="1"/>
+    <row r="651" ht="14.25" customHeight="1"/>
+    <row r="652" ht="14.25" customHeight="1"/>
+    <row r="653" ht="14.25" customHeight="1"/>
+    <row r="654" ht="14.25" customHeight="1"/>
+    <row r="655" ht="14.25" customHeight="1"/>
+    <row r="656" ht="14.25" customHeight="1"/>
+    <row r="657" ht="14.25" customHeight="1"/>
+    <row r="658" ht="14.25" customHeight="1"/>
+    <row r="659" ht="14.25" customHeight="1"/>
+    <row r="660" ht="14.25" customHeight="1"/>
+    <row r="661" ht="14.25" customHeight="1"/>
+    <row r="662" ht="14.25" customHeight="1"/>
+    <row r="663" ht="14.25" customHeight="1"/>
+    <row r="664" ht="14.25" customHeight="1"/>
+    <row r="665" ht="14.25" customHeight="1"/>
+    <row r="666" ht="14.25" customHeight="1"/>
+    <row r="667" ht="14.25" customHeight="1"/>
+    <row r="668" ht="14.25" customHeight="1"/>
+    <row r="669" ht="14.25" customHeight="1"/>
+    <row r="670" ht="14.25" customHeight="1"/>
+    <row r="671" ht="14.25" customHeight="1"/>
+    <row r="672" ht="14.25" customHeight="1"/>
+    <row r="673" ht="14.25" customHeight="1"/>
+    <row r="674" ht="14.25" customHeight="1"/>
+    <row r="675" ht="14.25" customHeight="1"/>
+    <row r="676" ht="14.25" customHeight="1"/>
+    <row r="677" ht="14.25" customHeight="1"/>
+    <row r="678" ht="14.25" customHeight="1"/>
+    <row r="679" ht="14.25" customHeight="1"/>
+    <row r="680" ht="14.25" customHeight="1"/>
+    <row r="681" ht="14.25" customHeight="1"/>
+    <row r="682" ht="14.25" customHeight="1"/>
+    <row r="683" ht="14.25" customHeight="1"/>
+    <row r="684" ht="14.25" customHeight="1"/>
+    <row r="685" ht="14.25" customHeight="1"/>
+    <row r="686" ht="14.25" customHeight="1"/>
+    <row r="687" ht="14.25" customHeight="1"/>
+    <row r="688" ht="14.25" customHeight="1"/>
+    <row r="689" ht="14.25" customHeight="1"/>
+    <row r="690" ht="14.25" customHeight="1"/>
+    <row r="691" ht="14.25" customHeight="1"/>
+    <row r="692" ht="14.25" customHeight="1"/>
+    <row r="693" ht="14.25" customHeight="1"/>
+    <row r="694" ht="14.25" customHeight="1"/>
+    <row r="695" ht="14.25" customHeight="1"/>
+    <row r="696" ht="14.25" customHeight="1"/>
+    <row r="697" ht="14.25" customHeight="1"/>
+    <row r="698" ht="14.25" customHeight="1"/>
+    <row r="699" ht="14.25" customHeight="1"/>
+    <row r="700" ht="14.25" customHeight="1"/>
+    <row r="701" ht="14.25" customHeight="1"/>
+    <row r="702" ht="14.25" customHeight="1"/>
+    <row r="703" ht="14.25" customHeight="1"/>
+    <row r="704" ht="14.25" customHeight="1"/>
+    <row r="705" ht="14.25" customHeight="1"/>
+    <row r="706" ht="14.25" customHeight="1"/>
+    <row r="707" ht="14.25" customHeight="1"/>
+    <row r="708" ht="14.25" customHeight="1"/>
+    <row r="709" ht="14.25" customHeight="1"/>
+    <row r="710" ht="14.25" customHeight="1"/>
+    <row r="711" ht="14.25" customHeight="1"/>
+    <row r="712" ht="14.25" customHeight="1"/>
+    <row r="713" ht="14.25" customHeight="1"/>
+    <row r="714" ht="14.25" customHeight="1"/>
+    <row r="715" ht="14.25" customHeight="1"/>
+    <row r="716" ht="14.25" customHeight="1"/>
+    <row r="717" ht="14.25" customHeight="1"/>
+    <row r="718" ht="14.25" customHeight="1"/>
+    <row r="719" ht="14.25" customHeight="1"/>
+    <row r="720" ht="14.25" customHeight="1"/>
+    <row r="721" ht="14.25" customHeight="1"/>
+    <row r="722" ht="14.25" customHeight="1"/>
+    <row r="723" ht="14.25" customHeight="1"/>
+    <row r="724" ht="14.25" customHeight="1"/>
+    <row r="725" ht="14.25" customHeight="1"/>
+    <row r="726" ht="14.25" customHeight="1"/>
+    <row r="727" ht="14.25" customHeight="1"/>
+    <row r="728" ht="14.25" customHeight="1"/>
+    <row r="729" ht="14.25" customHeight="1"/>
+    <row r="730" ht="14.25" customHeight="1"/>
+    <row r="731" ht="14.25" customHeight="1"/>
+    <row r="732" ht="14.25" customHeight="1"/>
+    <row r="733" ht="14.25" customHeight="1"/>
+    <row r="734" ht="14.25" customHeight="1"/>
+    <row r="735" ht="14.25" customHeight="1"/>
+    <row r="736" ht="14.25" customHeight="1"/>
+    <row r="737" ht="14.25" customHeight="1"/>
+    <row r="738" ht="14.25" customHeight="1"/>
+    <row r="739" ht="14.25" customHeight="1"/>
+    <row r="740" ht="14.25" customHeight="1"/>
+    <row r="741" ht="14.25" customHeight="1"/>
+    <row r="742" ht="14.25" customHeight="1"/>
+    <row r="743" ht="14.25" customHeight="1"/>
+    <row r="744" ht="14.25" customHeight="1"/>
+    <row r="745" ht="14.25" customHeight="1"/>
+    <row r="746" ht="14.25" customHeight="1"/>
+    <row r="747" ht="14.25" customHeight="1"/>
+    <row r="748" ht="14.25" customHeight="1"/>
+    <row r="749" ht="14.25" customHeight="1"/>
+    <row r="750" ht="14.25" customHeight="1"/>
+    <row r="751" ht="14.25" customHeight="1"/>
+    <row r="752" ht="14.25" customHeight="1"/>
+    <row r="753" ht="14.25" customHeight="1"/>
+    <row r="754" ht="14.25" customHeight="1"/>
+    <row r="755" ht="14.25" customHeight="1"/>
+    <row r="756" ht="14.25" customHeight="1"/>
+    <row r="757" ht="14.25" customHeight="1"/>
+    <row r="758" ht="14.25" customHeight="1"/>
+    <row r="759" ht="14.25" customHeight="1"/>
+    <row r="760" ht="14.25" customHeight="1"/>
+    <row r="761" ht="14.25" customHeight="1"/>
+    <row r="762" ht="14.25" customHeight="1"/>
+    <row r="763" ht="14.25" customHeight="1"/>
+    <row r="764" ht="14.25" customHeight="1"/>
+    <row r="765" ht="14.25" customHeight="1"/>
+    <row r="766" ht="14.25" customHeight="1"/>
+    <row r="767" ht="14.25" customHeight="1"/>
+    <row r="768" ht="14.25" customHeight="1"/>
+    <row r="769" ht="14.25" customHeight="1"/>
+    <row r="770" ht="14.25" customHeight="1"/>
+    <row r="771" ht="14.25" customHeight="1"/>
+    <row r="772" ht="14.25" customHeight="1"/>
+    <row r="773" ht="14.25" customHeight="1"/>
+    <row r="774" ht="14.25" customHeight="1"/>
+    <row r="775" ht="14.25" customHeight="1"/>
+    <row r="776" ht="14.25" customHeight="1"/>
+    <row r="777" ht="14.25" customHeight="1"/>
+    <row r="778" ht="14.25" customHeight="1"/>
+    <row r="779" ht="14.25" customHeight="1"/>
+    <row r="780" ht="14.25" customHeight="1"/>
+    <row r="781" ht="14.25" customHeight="1"/>
+    <row r="782" ht="14.25" customHeight="1"/>
+    <row r="783" ht="14.25" customHeight="1"/>
+    <row r="784" ht="14.25" customHeight="1"/>
+    <row r="785" ht="14.25" customHeight="1"/>
+    <row r="786" ht="14.25" customHeight="1"/>
+    <row r="787" ht="14.25" customHeight="1"/>
+    <row r="788" ht="14.25" customHeight="1"/>
+    <row r="789" ht="14.25" customHeight="1"/>
+    <row r="790" ht="14.25" customHeight="1"/>
+    <row r="791" ht="14.25" customHeight="1"/>
+    <row r="792" ht="14.25" customHeight="1"/>
+    <row r="793" ht="14.25" customHeight="1"/>
+    <row r="794" ht="14.25" customHeight="1"/>
+    <row r="795" ht="14.25" customHeight="1"/>
+    <row r="796" ht="14.25" customHeight="1"/>
+    <row r="797" ht="14.25" customHeight="1"/>
+    <row r="798" ht="14.25" customHeight="1"/>
+    <row r="799" ht="14.25" customHeight="1"/>
+    <row r="800" ht="14.25" customHeight="1"/>
+    <row r="801" ht="14.25" customHeight="1"/>
+    <row r="802" ht="14.25" customHeight="1"/>
+    <row r="803" ht="14.25" customHeight="1"/>
+    <row r="804" ht="14.25" customHeight="1"/>
+    <row r="805" ht="14.25" customHeight="1"/>
+    <row r="806" ht="14.25" customHeight="1"/>
+    <row r="807" ht="14.25" customHeight="1"/>
+    <row r="808" ht="14.25" customHeight="1"/>
+    <row r="809" ht="14.25" customHeight="1"/>
+    <row r="810" ht="14.25" customHeight="1"/>
+    <row r="811" ht="14.25" customHeight="1"/>
+    <row r="812" ht="14.25" customHeight="1"/>
+    <row r="813" ht="14.25" customHeight="1"/>
+    <row r="814" ht="14.25" customHeight="1"/>
+    <row r="815" ht="14.25" customHeight="1"/>
+    <row r="816" ht="14.25" customHeight="1"/>
+    <row r="817" ht="14.25" customHeight="1"/>
+    <row r="818" ht="14.25" customHeight="1"/>
+    <row r="819" ht="14.25" customHeight="1"/>
+    <row r="820" ht="14.25" customHeight="1"/>
+    <row r="821" ht="14.25" customHeight="1"/>
+    <row r="822" ht="14.25" customHeight="1"/>
+    <row r="823" ht="14.25" customHeight="1"/>
+    <row r="824" ht="14.25" customHeight="1"/>
+    <row r="825" ht="14.25" customHeight="1"/>
+    <row r="826" ht="14.25" customHeight="1"/>
+    <row r="827" ht="14.25" customHeight="1"/>
+    <row r="828" ht="14.25" customHeight="1"/>
+    <row r="829" ht="14.25" customHeight="1"/>
+    <row r="830" ht="14.25" customHeight="1"/>
+    <row r="831" ht="14.25" customHeight="1"/>
+    <row r="832" ht="14.25" customHeight="1"/>
+    <row r="833" ht="14.25" customHeight="1"/>
+    <row r="834" ht="14.25" customHeight="1"/>
+    <row r="835" ht="14.25" customHeight="1"/>
+    <row r="836" ht="14.25" customHeight="1"/>
+    <row r="837" ht="14.25" customHeight="1"/>
+    <row r="838" ht="14.25" customHeight="1"/>
+    <row r="839" ht="14.25" customHeight="1"/>
+    <row r="840" ht="14.25" customHeight="1"/>
+    <row r="841" ht="14.25" customHeight="1"/>
+    <row r="842" ht="14.25" customHeight="1"/>
+    <row r="843" ht="14.25" customHeight="1"/>
+    <row r="844" ht="14.25" customHeight="1"/>
+    <row r="845" ht="14.25" customHeight="1"/>
+    <row r="846" ht="14.25" customHeight="1"/>
+    <row r="847" ht="14.25" customHeight="1"/>
+    <row r="848" ht="14.25" customHeight="1"/>
+    <row r="849" ht="14.25" customHeight="1"/>
+    <row r="850" ht="14.25" customHeight="1"/>
+    <row r="851" ht="14.25" customHeight="1"/>
+    <row r="852" ht="14.25" customHeight="1"/>
+    <row r="853" ht="14.25" customHeight="1"/>
+    <row r="854" ht="14.25" customHeight="1"/>
+    <row r="855" ht="14.25" customHeight="1"/>
+    <row r="856" ht="14.25" customHeight="1"/>
+    <row r="857" ht="14.25" customHeight="1"/>
+    <row r="858" ht="14.25" customHeight="1"/>
+    <row r="859" ht="14.25" customHeight="1"/>
+    <row r="860" ht="14.25" customHeight="1"/>
+    <row r="861" ht="14.25" customHeight="1"/>
+    <row r="862" ht="14.25" customHeight="1"/>
+    <row r="863" ht="14.25" customHeight="1"/>
+    <row r="864" ht="14.25" customHeight="1"/>
+    <row r="865" ht="14.25" customHeight="1"/>
+    <row r="866" ht="14.25" customHeight="1"/>
+    <row r="867" ht="14.25" customHeight="1"/>
+    <row r="868" ht="14.25" customHeight="1"/>
+    <row r="869" ht="14.25" customHeight="1"/>
+    <row r="870" ht="14.25" customHeight="1"/>
+    <row r="871" ht="14.25" customHeight="1"/>
+    <row r="872" ht="14.25" customHeight="1"/>
+    <row r="873" ht="14.25" customHeight="1"/>
+    <row r="874" ht="14.25" customHeight="1"/>
+    <row r="875" ht="14.25" customHeight="1"/>
+    <row r="876" ht="14.25" customHeight="1"/>
+    <row r="877" ht="14.25" customHeight="1"/>
+    <row r="878" ht="14.25" customHeight="1"/>
+    <row r="879" ht="14.25" customHeight="1"/>
+    <row r="880" ht="14.25" customHeight="1"/>
+    <row r="881" ht="14.25" customHeight="1"/>
+    <row r="882" ht="14.25" customHeight="1"/>
+    <row r="883" ht="14.25" customHeight="1"/>
+    <row r="884" ht="14.25" customHeight="1"/>
+    <row r="885" ht="14.25" customHeight="1"/>
+    <row r="886" ht="14.25" customHeight="1"/>
+    <row r="887" ht="14.25" customHeight="1"/>
+    <row r="888" ht="14.25" customHeight="1"/>
+    <row r="889" ht="14.25" customHeight="1"/>
+    <row r="890" ht="14.25" customHeight="1"/>
+    <row r="891" ht="14.25" customHeight="1"/>
+    <row r="892" ht="14.25" customHeight="1"/>
+    <row r="893" ht="14.25" customHeight="1"/>
+    <row r="894" ht="14.25" customHeight="1"/>
+    <row r="895" ht="14.25" customHeight="1"/>
+    <row r="896" ht="14.25" customHeight="1"/>
+    <row r="897" ht="14.25" customHeight="1"/>
+    <row r="898" ht="14.25" customHeight="1"/>
+    <row r="899" ht="14.25" customHeight="1"/>
+    <row r="900" ht="14.25" customHeight="1"/>
+    <row r="901" ht="14.25" customHeight="1"/>
+    <row r="902" ht="14.25" customHeight="1"/>
+    <row r="903" ht="14.25" customHeight="1"/>
+    <row r="904" ht="14.25" customHeight="1"/>
+    <row r="905" ht="14.25" customHeight="1"/>
+    <row r="906" ht="14.25" customHeight="1"/>
+    <row r="907" ht="14.25" customHeight="1"/>
+    <row r="908" ht="14.25" customHeight="1"/>
+    <row r="909" ht="14.25" customHeight="1"/>
+    <row r="910" ht="14.25" customHeight="1"/>
+    <row r="911" ht="14.25" customHeight="1"/>
+    <row r="912" ht="14.25" customHeight="1"/>
+    <row r="913" ht="14.25" customHeight="1"/>
+    <row r="914" ht="14.25" customHeight="1"/>
+    <row r="915" ht="14.25" customHeight="1"/>
+    <row r="916" ht="14.25" customHeight="1"/>
+    <row r="917" ht="14.25" customHeight="1"/>
+    <row r="918" ht="14.25" customHeight="1"/>
+    <row r="919" ht="14.25" customHeight="1"/>
+    <row r="920" ht="14.25" customHeight="1"/>
+    <row r="921" ht="14.25" customHeight="1"/>
+    <row r="922" ht="14.25" customHeight="1"/>
+    <row r="923" ht="14.25" customHeight="1"/>
+    <row r="924" ht="14.25" customHeight="1"/>
+    <row r="925" ht="14.25" customHeight="1"/>
+    <row r="926" ht="14.25" customHeight="1"/>
+    <row r="927" ht="14.25" customHeight="1"/>
+    <row r="928" ht="14.25" customHeight="1"/>
+    <row r="929" ht="14.25" customHeight="1"/>
+    <row r="930" ht="14.25" customHeight="1"/>
+    <row r="931" ht="14.25" customHeight="1"/>
+    <row r="932" ht="14.25" customHeight="1"/>
+    <row r="933" ht="14.25" customHeight="1"/>
+    <row r="934" ht="14.25" customHeight="1"/>
+    <row r="935" ht="14.25" customHeight="1"/>
+    <row r="936" ht="14.25" customHeight="1"/>
+    <row r="937" ht="14.25" customHeight="1"/>
+    <row r="938" ht="14.25" customHeight="1"/>
+    <row r="939" ht="14.25" customHeight="1"/>
+    <row r="940" ht="14.25" customHeight="1"/>
+    <row r="941" ht="14.25" customHeight="1"/>
+    <row r="942" ht="14.25" customHeight="1"/>
+    <row r="943" ht="14.25" customHeight="1"/>
+    <row r="944" ht="14.25" customHeight="1"/>
+    <row r="945" ht="14.25" customHeight="1"/>
+    <row r="946" ht="14.25" customHeight="1"/>
+    <row r="947" ht="14.25" customHeight="1"/>
+    <row r="948" ht="14.25" customHeight="1"/>
+    <row r="949" ht="14.25" customHeight="1"/>
+    <row r="950" ht="14.25" customHeight="1"/>
+    <row r="951" ht="14.25" customHeight="1"/>
+    <row r="952" ht="14.25" customHeight="1"/>
+    <row r="953" ht="14.25" customHeight="1"/>
+    <row r="954" ht="14.25" customHeight="1"/>
+    <row r="955" ht="14.25" customHeight="1"/>
+    <row r="956" ht="14.25" customHeight="1"/>
+    <row r="957" ht="14.25" customHeight="1"/>
+    <row r="958" ht="14.25" customHeight="1"/>
+    <row r="959" ht="14.25" customHeight="1"/>
+    <row r="960" ht="14.25" customHeight="1"/>
+    <row r="961" ht="14.25" customHeight="1"/>
+    <row r="962" ht="14.25" customHeight="1"/>
+    <row r="963" ht="14.25" customHeight="1"/>
+    <row r="964" ht="14.25" customHeight="1"/>
+    <row r="965" ht="14.25" customHeight="1"/>
+    <row r="966" ht="14.25" customHeight="1"/>
+    <row r="967" ht="14.25" customHeight="1"/>
+    <row r="968" ht="14.25" customHeight="1"/>
+    <row r="969" ht="14.25" customHeight="1"/>
+    <row r="970" ht="14.25" customHeight="1"/>
+    <row r="971" ht="14.25" customHeight="1"/>
+    <row r="972" ht="14.25" customHeight="1"/>
+    <row r="973" ht="14.25" customHeight="1"/>
+    <row r="974" ht="14.25" customHeight="1"/>
+    <row r="975" ht="14.25" customHeight="1"/>
+    <row r="976" ht="14.25" customHeight="1"/>
+    <row r="977" ht="14.25" customHeight="1"/>
+    <row r="978" ht="14.25" customHeight="1"/>
+    <row r="979" ht="14.25" customHeight="1"/>
+    <row r="980" ht="14.25" customHeight="1"/>
+    <row r="981" ht="14.25" customHeight="1"/>
+    <row r="982" ht="14.25" customHeight="1"/>
+    <row r="983" ht="14.25" customHeight="1"/>
+    <row r="984" ht="14.25" customHeight="1"/>
+    <row r="985" ht="14.25" customHeight="1"/>
+    <row r="986" ht="14.25" customHeight="1"/>
+    <row r="987" ht="14.25" customHeight="1"/>
+    <row r="988" ht="14.25" customHeight="1"/>
+    <row r="989" ht="14.25" customHeight="1"/>
+    <row r="990" ht="14.25" customHeight="1"/>
+    <row r="991" ht="14.25" customHeight="1"/>
+    <row r="992" ht="14.25" customHeight="1"/>
+    <row r="993" ht="14.25" customHeight="1"/>
+    <row r="994" ht="14.25" customHeight="1"/>
+    <row r="995" ht="14.25" customHeight="1"/>
+    <row r="996" ht="14.25" customHeight="1"/>
+    <row r="997" ht="14.25" customHeight="1"/>
+    <row r="998" ht="14.25" customHeight="1"/>
+    <row r="999" ht="14.25" customHeight="1"/>
+    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <printOptions/>
+  <pageMargins bottom="0.787401575" footer="0.0" header="0.0" left="0.511811024" right="0.511811024" top="0.787401575"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>